<commit_message>
feat(cards): implement Kanji lookup modal, font catalog assets, and UI refinements
</commit_message>
<xml_diff>
--- a/app/src/main/assets/kotoba_deck_template.xlsx
+++ b/app/src/main/assets/kotoba_deck_template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Kotoba Deck" sheetId="1" r:id="rId1"/>
+    <sheet name="Koto Deck" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -13,7 +13,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Japanese / Kana</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -33,7 +33,22 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Context / Notes</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Example 1 (JP &amp; EN)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Example 2 (JP &amp; EN)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Example 3 (JP &amp; EN)</t>
         </is>
       </c>
     </row>
@@ -60,7 +75,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Healthcare / Facilities</t>
+          <t>Essential healthcare vocabulary; used when visiting medical facilities.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>明日、病院に行きます。 / I will go to the hospital tomorrow.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>病院の前に薬局があります。 / There is a pharmacy in front of the hospital.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>近くに大きな病院がありますか？ / Is there a large hospital nearby?</t>
         </is>
       </c>
     </row>
@@ -87,7 +117,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Group 2 verb</t>
+          <t>Group 2 (ichidan) verb; versatile base verb for dining and meals.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>朝ごはんを食べましたか？ / Did you eat breakfast?</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>日本料理を美味しく食べる。 / To eat Japanese food deliciously.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>一緒にお昼ご飯を食べましょう。 / Let's eat lunch together.</t>
         </is>
       </c>
     </row>
@@ -114,7 +159,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Casual expression</t>
+          <t>Everyday polite gratitude expression; often expanded to 'ありがとうございます'.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>手伝ってくれてありがとう。 / Thank you for helping me.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>プレゼントを本当にありがとう。 / Thank you so much for the present.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>いつも温かい言葉をありがとう。 / Thank you always for your warm words.</t>
         </is>
       </c>
     </row>

</xml_diff>